<commit_message>
Added paper information, added Research Methodology section to paper
</commit_message>
<xml_diff>
--- a/paper_information.xlsx
+++ b/paper_information.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agi\Documents\_ELTE\_MSc\DSLab\DS-Lab-AI-Security-Ontology\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2B94BED-AEF6-4076-976A-0A996CD3B024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1FCBB5-EA31-48F0-A87D-11FC22D96D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Literature - 1st Milestone" sheetId="1" r:id="rId1"/>
+    <sheet name="Literature using LLMs" sheetId="2" r:id="rId1"/>
+    <sheet name="Literature not using LLMs" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="53">
   <si>
     <t>Title</t>
   </si>
@@ -42,30 +43,426 @@
     <t>Ontology Development Methodology: A Systematic Review and Case Study</t>
   </si>
   <si>
-    <t>2022 2nd International Conference on Computing and Information Technology (ICCIT)</t>
-  </si>
-  <si>
     <t>Methods</t>
   </si>
   <si>
-    <t>data was extracted from the website of University of Tabuk (https://www.ut.edu.sa/ar/Faculties/computer-and-information-technology/
-Department-Information-Technology/Pages/study-plans.aspx)</t>
-  </si>
-  <si>
-    <t>following the steps of Simple Knowledge-Engineering Methodology</t>
-  </si>
-  <si>
-    <t>evaluation, test the competency of the ontology and maintenance were not included, only mentioned for future work</t>
-  </si>
-  <si>
     <t>#</t>
+  </si>
+  <si>
+    <t>An Ontological Knowledge Base of Poisoning Attacks on Deep Neural Networks</t>
+  </si>
+  <si>
+    <t>Institute of Electrical and Electronics Engineers Inc.</t>
+  </si>
+  <si>
+    <t>Applied Sciences (Switzerland)</t>
+  </si>
+  <si>
+    <r>
+      <t>Phase 1: Systematic</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Literature Review                 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Phase 2: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Taxonomy </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Extracting                                Phase 3: Developing DNNPAO (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>knowledge base</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>Tools</t>
+  </si>
+  <si>
+    <t>Great introduction structure, informative graphs, mentions automation tools for SLR, clever class definitions</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Data was extracted from research papers listed in SLR                                             GitHub: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="8"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://github.com/MajedCS/DNNPAO</t>
+    </r>
+  </si>
+  <si>
+    <t>Simple Knowledge-Engineering Methodology</t>
+  </si>
+  <si>
+    <t>Evaluation, test the competency of the ontology and maintenance were not included, only mentioned for future work</t>
+  </si>
+  <si>
+    <t>Only focuses on poisoning attacks (during training and testing phase) against DDNs, relatively small number of nodes, and therefore performance and scalability were not main concerns</t>
+  </si>
+  <si>
+    <r>
+      <t>Data was extracted from the website of University of Tabuk (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="8"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://www.ut.edu.sa/ar/Faculties/computer-and-information-technology/Department-Information-Technology/Pages/study-plans.aspx</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>The Artiﬁcial Intelligence Ontology: LLM-Assisted Construction of AI Concept Hierarchies</t>
+  </si>
+  <si>
+    <t>Applied Ontology</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>From human experts to machines: An LLM supported approach to ontology and knowledge graph construction</t>
+  </si>
+  <si>
+    <t>2024.03.13.</t>
+  </si>
+  <si>
+    <t>License</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">CC BY NC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="8"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://www.sagepub.com/journals/permissions/pre-approved-permission-requests?_gl=1*1m753mr*_up*MQ..*_ga*MzA0MTMwNTI5LjE3NzYxODk4OTE.*_ga_60R758KFDG*czE3NzYxODk4OTEkbzEkZzAkdDE3NzYxODk4OTEkajYwJGwwJGgxNDM2MzA0ODY5</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">CC BY </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="8"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://creativecommons.org/licenses/by/4.0/</t>
+    </r>
+  </si>
+  <si>
+    <t>Accelerating knowledge graph and ontology engineering with large language models</t>
+  </si>
+  <si>
+    <t>2025.05.01.</t>
+  </si>
+  <si>
+    <t>Journal of Web Semantics</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">CC BY-NC-ND </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="8"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://creativecommons.org/licenses/by-nc-nd/4.0/</t>
+    </r>
+  </si>
+  <si>
+    <t>An LLM supported approach to ontology and knowledge graph construction</t>
+  </si>
+  <si>
+    <t>Authorized licensed use limited to: Eotvos Lorand University Budapest. Downloaded on March 25,2026 at 15:50:08 UTC from IEEE Xplore. Restrictions apply.</t>
+  </si>
+  <si>
+    <t>Authorized licensed use limited to: Eotvos Lorand University Budapest. Downloaded on March 11,2026 at 21:47:37 UTC from IEEE Xplore. Restrictions apply.</t>
+  </si>
+  <si>
+    <t>PubMed, Scholarly Publications</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Created </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>initial ontology</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (by human based on literature) </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>LLM created CQs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and ontology was expanded by it    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>LLM answered CQs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and used the ontology to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>create KG</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>OWL + Portégé</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, webportege.standford.edu, Neo4j GD, Neosemantics plugin</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Portégé, ChatGPT-3.5 fine tuned </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>on breast cancer treatment guidelines and related literature to fine</t>
+    </r>
+  </si>
+  <si>
+    <t>Evaluation is done by LLM                                                                                 They mention iterative CQ generation and KG update for future work</t>
+  </si>
+  <si>
+    <t>Terms like Ontology, KG, LLM nicely introduced, informative graph about Methods</t>
+  </si>
+  <si>
+    <t>No data was used</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Modular Ontology Modeling</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (MOMo)                                     - ontology modeling, extension and modification                       - ontology alignment                                                                      - ontology population + entity disambiguation</t>
+    </r>
+  </si>
+  <si>
+    <t>More industrial/business use case than research (?)</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Portégé</t>
+  </si>
+  <si>
+    <t>CoModIDE for MOMo, OPLa expressed in OWL, ODP libraries, Portégé plugin</t>
+  </si>
+  <si>
+    <t>Many citations of previous work, article not so informative, doesn't describe method in detail nor provide specific use case</t>
+  </si>
+  <si>
+    <t>2024.11.16.</t>
+  </si>
+  <si>
+    <t>Ontology Development Kit (ODK), Claude 3 Sonnet, GPT-4, ROBOT-helper chatbot</t>
+  </si>
+  <si>
+    <t>2022.11.</t>
+  </si>
+  <si>
+    <t>Publications, Wikipedia, documentations</t>
+  </si>
+  <si>
+    <t>ROBOT templates + manual creation of branches  populated both manually and automatically                LLMs were used to improve definitions, final definitions were human-reviewed</t>
+  </si>
+  <si>
+    <t>CC BY https://creativecommons.org/licenses/by/4.0/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -77,6 +474,28 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -108,7 +527,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -125,9 +544,42 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normál" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -404,60 +856,290 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:F3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDB31F52-68CC-4180-96AF-48F199FC4213}">
+  <dimension ref="A2:J13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.6640625" customWidth="1"/>
-    <col min="2" max="2" width="34.88671875" customWidth="1"/>
-    <col min="3" max="3" width="43.77734375" customWidth="1"/>
-    <col min="4" max="4" width="69.44140625" customWidth="1"/>
-    <col min="5" max="5" width="37.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="57.109375" customWidth="1"/>
+    <col min="1" max="1" width="3.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="11.5546875" style="9" customWidth="1"/>
+    <col min="3" max="3" width="35.33203125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="43.77734375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="69.44140625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="46.109375" style="6" customWidth="1"/>
+    <col min="7" max="7" width="57.109375" style="6" customWidth="1"/>
+    <col min="8" max="8" width="40.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="44.33203125" style="6" customWidth="1"/>
+    <col min="10" max="10" width="39.21875" style="6" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="F2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="H2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="10">
+        <v>2024</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="59.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>3</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="H5" s="4"/>
+      <c r="I5" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" s="16" customFormat="1" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="11">
         <v>4</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="B6" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="14"/>
+      <c r="J6" s="16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C13" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A2:J4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.6640625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="11" style="6" customWidth="1"/>
+    <col min="3" max="3" width="34.88671875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="43.77734375" style="6" customWidth="1"/>
+    <col min="5" max="5" width="69.44140625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="43.5546875" style="6" customWidth="1"/>
+    <col min="7" max="7" width="57.109375" style="6" customWidth="1"/>
+    <col min="8" max="8" width="40.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="44.33203125" style="6" customWidth="1"/>
+    <col min="10" max="10" width="39.21875" style="6" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="10">
+        <v>2022</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>